<commit_message>
chore: 更新 now/MHXY.xlsx 数据
Co-Authored-By: AtomCode (grok-4.5) <noreply@atomgit.com>
</commit_message>
<xml_diff>
--- a/now/MHXY.xlsx
+++ b/now/MHXY.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\MHH\now\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="13560" windowHeight="7485" activeTab="2"/>
+    <workbookView windowWidth="28800" windowHeight="12375" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="支出明细表" sheetId="1" r:id="rId1"/>
@@ -29,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="97">
   <si>
     <t>梦幻西游 · 支出明细表（黄色行为新增录入区）</t>
   </si>
@@ -154,6 +159,9 @@
     <t>力宠龙鲤</t>
   </si>
   <si>
+    <t>力宠 （已卖出）</t>
+  </si>
+  <si>
     <t>购入法宠</t>
   </si>
   <si>
@@ -224,6 +232,12 @@
   </si>
   <si>
     <t>采购法宠卖出收入</t>
+  </si>
+  <si>
+    <t>龙鲤</t>
+  </si>
+  <si>
+    <t>卖出</t>
   </si>
   <si>
     <t>宠物小计</t>
@@ -323,7 +337,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -389,13 +403,6 @@
       <color rgb="FFC00000"/>
       <name val="微软雅黑"/>
       <charset val="134"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <u/>
@@ -902,148 +909,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="10" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1848,7 +1855,7 @@
         <v>168</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
     </row>
     <row r="35" ht="16.5" spans="1:4">
@@ -1856,13 +1863,13 @@
         <v>35</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C35" s="8">
         <v>106</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="36" ht="16.5" spans="1:4">
@@ -1910,19 +1917,19 @@
         <v>15</v>
       </c>
       <c r="B41" s="20" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C41" s="21">
         <f>SUM(C31:C40)</f>
         <v>662</v>
       </c>
       <c r="D41" s="20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="42" ht="26" customHeight="1" spans="1:4">
       <c r="A42" s="16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B42" s="17"/>
       <c r="C42" s="17"/>
@@ -1930,49 +1937,49 @@
     </row>
     <row r="43" ht="16.5" spans="1:4">
       <c r="A43" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C43" s="8">
         <v>20</v>
       </c>
       <c r="D43" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44" ht="16.5" spans="1:4">
       <c r="A44" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C44" s="8">
         <v>35</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="45" ht="16.5" spans="1:4">
       <c r="A45" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C45" s="8">
         <v>40.5</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="46" ht="16.5" spans="1:4">
       <c r="A46" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B46" s="18"/>
       <c r="C46" s="19"/>
@@ -1980,7 +1987,7 @@
     </row>
     <row r="47" ht="16.5" spans="1:4">
       <c r="A47" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B47" s="18"/>
       <c r="C47" s="19"/>
@@ -1988,7 +1995,7 @@
     </row>
     <row r="48" ht="16.5" spans="1:4">
       <c r="A48" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B48" s="18"/>
       <c r="C48" s="19"/>
@@ -1996,7 +2003,7 @@
     </row>
     <row r="49" ht="16.5" spans="1:4">
       <c r="A49" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B49" s="18"/>
       <c r="C49" s="19"/>
@@ -2004,7 +2011,7 @@
     </row>
     <row r="50" ht="16.5" spans="1:4">
       <c r="A50" s="18" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B50" s="18"/>
       <c r="C50" s="19"/>
@@ -2015,14 +2022,14 @@
         <v>15</v>
       </c>
       <c r="B51" s="20" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C51" s="21">
         <f>SUM(C43:C50)</f>
         <v>95.5</v>
       </c>
       <c r="D51" s="20" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="53" ht="18" spans="1:4">
@@ -2030,24 +2037,24 @@
         <v>15</v>
       </c>
       <c r="B53" s="22" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C53" s="11">
         <f>C14+C29+C41+C51</f>
         <v>3959.4</v>
       </c>
       <c r="D53" s="22" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="55" ht="16.5" spans="1:4">
       <c r="A55" s="14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="56" ht="16.5" spans="1:4">
       <c r="A56" s="14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -2079,15 +2086,15 @@
   <sheetData>
     <row r="1" ht="38" customHeight="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:4">
       <c r="A2" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>3</v>
@@ -2098,7 +2105,7 @@
     </row>
     <row r="3" ht="26" customHeight="1" spans="1:4">
       <c r="A3" s="16" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B3" s="17"/>
       <c r="C3" s="17"/>
@@ -2106,29 +2113,35 @@
     </row>
     <row r="4" ht="16.5" spans="1:4">
       <c r="A4" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C4" s="8">
         <v>85.5</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" ht="16.5" spans="1:4">
       <c r="A5" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5" s="18"/>
-      <c r="C5" s="19"/>
-      <c r="D5" s="18"/>
+        <v>63</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="19">
+        <v>161.5</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="6" ht="16.5" spans="1:4">
       <c r="A6" s="18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B6" s="18"/>
       <c r="C6" s="19"/>
@@ -2136,7 +2149,7 @@
     </row>
     <row r="7" ht="16.5" spans="1:4">
       <c r="A7" s="18" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B7" s="18"/>
       <c r="C7" s="19"/>
@@ -2147,11 +2160,11 @@
         <v>15</v>
       </c>
       <c r="B8" s="20" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C8" s="21">
         <f>SUM(C4:C7)</f>
-        <v>85.5</v>
+        <v>247</v>
       </c>
       <c r="D8" s="20" t="s">
         <v>15</v>
@@ -2159,7 +2172,7 @@
     </row>
     <row r="9" ht="26" customHeight="1" spans="1:4">
       <c r="A9" s="16" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B9" s="17"/>
       <c r="C9" s="17"/>
@@ -2167,77 +2180,77 @@
     </row>
     <row r="10" ht="16.5" spans="1:4">
       <c r="A10" s="9" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C10" s="8">
         <v>202</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" ht="16.5" spans="1:4">
       <c r="A11" s="9" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C11" s="8">
         <v>67.45</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" ht="16.5" spans="1:4">
       <c r="A12" s="9" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C12" s="8">
         <v>67.45</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" ht="16.5" spans="1:4">
       <c r="A13" s="9" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C13" s="8">
         <v>66.78</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" ht="16.5" spans="1:4">
       <c r="A14" s="9" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C14" s="8">
         <v>66.78</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" ht="16.5" spans="1:4">
       <c r="A15" s="18" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B15" s="18"/>
       <c r="C15" s="19"/>
@@ -2245,7 +2258,7 @@
     </row>
     <row r="16" ht="16.5" spans="1:4">
       <c r="A16" s="18" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B16" s="18"/>
       <c r="C16" s="19"/>
@@ -2253,7 +2266,7 @@
     </row>
     <row r="17" ht="16.5" spans="1:4">
       <c r="A17" s="18" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B17" s="18"/>
       <c r="C17" s="19"/>
@@ -2261,7 +2274,7 @@
     </row>
     <row r="18" ht="16.5" spans="1:4">
       <c r="A18" s="18" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B18" s="18"/>
       <c r="C18" s="19"/>
@@ -2269,7 +2282,7 @@
     </row>
     <row r="19" ht="16.5" spans="1:4">
       <c r="A19" s="18" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B19" s="18"/>
       <c r="C19" s="19"/>
@@ -2280,7 +2293,7 @@
         <v>15</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C20" s="21">
         <f>SUM(C10:C19)</f>
@@ -2295,19 +2308,19 @@
         <v>15</v>
       </c>
       <c r="B22" s="22" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C22" s="11">
         <f>C8+C20</f>
-        <v>555.96</v>
+        <v>717.46</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" ht="16.5" spans="1:4">
       <c r="A24" s="14" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -2335,84 +2348,84 @@
   <sheetData>
     <row r="1" ht="38" customHeight="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" ht="28" customHeight="1" spans="1:3">
       <c r="A2" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" ht="16.5" spans="1:3">
       <c r="A3" s="4" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B3" s="5">
         <f>支出明细表!C53</f>
         <v>3959.4</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" ht="16.5" spans="1:3">
       <c r="A4" s="7" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B4" s="8">
         <f>游戏变现收入明细表!C22</f>
-        <v>555.96</v>
+        <v>717.46</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" ht="18" spans="1:3">
       <c r="A5" s="10" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B5" s="11">
         <f>B3-B4</f>
-        <v>3403.44</v>
+        <v>3241.94</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" ht="18" spans="1:3">
       <c r="A7" s="13" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:3">
       <c r="A8" s="14" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:3">
       <c r="A9" s="14" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:3">
       <c r="A10" s="14" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:3">
       <c r="A11" s="14" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:3">
       <c r="A12" s="14" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="14" ht="16.5" spans="1:3">

</xml_diff>